<commit_message>
-se actalizaron las rubricas de funcionalidad en ESP32 y Android con la version que se le entrego a los alumnos de SOA. -Además se agrego una rubrica de concurrencia en Ep32 que los docentes evaluen el código de esp32
</commit_message>
<xml_diff>
--- a/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultados Resumen metricas utilizadas 1C 2026.xlsx
+++ b/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultados Resumen metricas utilizadas 1C 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\Prog-Concurrente\Analisis de metricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E0C465-D30C-4BBA-90C1-B680C798917E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375AF90B-8CE7-4575-A71F-32E70E0CD7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -206,11 +206,6 @@
     <t>Claude Code</t>
   </si>
   <si>
-    <t>Haiku 4.5
-Sonnet 4.6 
-Opus 4.7</t>
-  </si>
-  <si>
     <t xml:space="preserve">Python en linux(backend)
 html y js(frontend)
 usa postgreSQL
@@ -1464,6 +1459,12 @@
 Con Claude Sonnet = 7418 tokens
 Con GPT = 5955 tokens
 Con Deepseek = 6670 tokens</t>
+  </si>
+  <si>
+    <t>Haiku 4.5
+Sonnet 4.6 
+Opus 4.7
+(todo junto)</t>
   </si>
 </sst>
 </file>
@@ -1638,10 +1639,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2116,167 +2116,167 @@
         <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H2" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="5" t="s">
+    <row r="3" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="H4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" s="6" t="s">
+      <c r="D6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C4" s="8" t="s">
+      <c r="G6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="D7" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="G7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>94</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2309,7 +2309,7 @@
       <c r="C1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -2317,783 +2317,783 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A3" s="14"/>
-      <c r="B3" s="15" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="17" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A4" s="38"/>
-      <c r="B4" s="17" t="s">
+      <c r="A4" s="37"/>
+      <c r="B4" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="19"/>
+      <c r="E4" s="18"/>
     </row>
     <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A5" s="38"/>
-      <c r="B5" s="17" t="s">
+      <c r="A5" s="37"/>
+      <c r="B5" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="19"/>
+      <c r="E5" s="18"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="38"/>
-      <c r="B6" s="17" t="s">
+      <c r="A6" s="37"/>
+      <c r="B6" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="19"/>
+      <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="38"/>
-      <c r="B7" s="17" t="s">
+      <c r="A7" s="37"/>
+      <c r="B7" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="19"/>
+      <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="38"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="37"/>
+      <c r="B8" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" s="18"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="37"/>
+      <c r="B9" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="18"/>
+    </row>
+    <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A10" s="38"/>
+      <c r="B10" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="23"/>
+      <c r="E10" s="24"/>
+    </row>
+    <row r="11" spans="1:5" ht="145" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="12"/>
+    </row>
+    <row r="12" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A12" s="13"/>
+      <c r="B12" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="17"/>
+    </row>
+    <row r="13" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="37"/>
+      <c r="B13" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="18"/>
+    </row>
+    <row r="14" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="37"/>
+      <c r="B14" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="18"/>
+    </row>
+    <row r="15" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A15" s="37"/>
+      <c r="B15" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="18"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="37"/>
+      <c r="B16" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="E16" s="18"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="37"/>
+      <c r="B17" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="18"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="37"/>
+      <c r="B18" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="18"/>
+    </row>
+    <row r="19" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A19" s="38"/>
+      <c r="B19" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E8" s="19"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="38"/>
-      <c r="B9" s="20" t="s">
+      <c r="E19" s="24"/>
+    </row>
+    <row r="20" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="13"/>
+      <c r="B21" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="27"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="17"/>
+    </row>
+    <row r="22" spans="1:5" ht="116" x14ac:dyDescent="0.35">
+      <c r="A22" s="37"/>
+      <c r="B22" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" s="18"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="37"/>
+      <c r="B23" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="18"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="37"/>
+      <c r="B24" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="18"/>
+    </row>
+    <row r="25" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A25" s="37"/>
+      <c r="B25" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25" s="18"/>
+    </row>
+    <row r="26" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A26" s="37"/>
+      <c r="B26" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="18"/>
+    </row>
+    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="37"/>
+      <c r="B27" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C27" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="20" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" s="19"/>
-    </row>
-    <row r="10" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" s="39"/>
-      <c r="B10" s="22" t="s">
+      <c r="D27" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="E27" s="18"/>
+    </row>
+    <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="38"/>
+      <c r="B28" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-    </row>
-    <row r="11" spans="1:5" ht="145" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="11" t="s">
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="24"/>
+    </row>
+    <row r="29" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="13"/>
-    </row>
-    <row r="12" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15" t="s">
+      <c r="C29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="30" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A30" s="13"/>
+      <c r="B30" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="28" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="18"/>
-    </row>
-    <row r="13" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="38"/>
-      <c r="B13" s="17" t="s">
+      <c r="C30" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="35" t="s">
+        <v>123</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A31" s="37"/>
+      <c r="B31" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="19"/>
-    </row>
-    <row r="14" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="38"/>
-      <c r="B14" s="17" t="s">
+      <c r="C31" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="E31" s="18"/>
+    </row>
+    <row r="32" spans="1:5" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="37"/>
+      <c r="B32" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="19"/>
-    </row>
-    <row r="15" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="38"/>
-      <c r="B15" s="17" t="s">
+      <c r="C32" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="D32" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="E32" s="18"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="37"/>
+      <c r="B33" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="19"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="38"/>
-      <c r="B16" s="17" t="s">
+      <c r="E33" s="18"/>
+    </row>
+    <row r="34" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A34" s="37"/>
+      <c r="B34" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D16" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="E16" s="19"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="38"/>
-      <c r="B17" s="20" t="s">
+      <c r="C34" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E34" s="18"/>
+    </row>
+    <row r="35" spans="1:5" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A35" s="37"/>
+      <c r="B35" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="19"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="38"/>
-      <c r="B18" s="20" t="s">
+      <c r="C35" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" s="18"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="37"/>
+      <c r="B36" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C36" s="20"/>
+      <c r="D36" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E36" s="18"/>
+    </row>
+    <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="38"/>
+      <c r="B37" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="20"/>
+      <c r="D37" s="20"/>
+      <c r="E37" s="24"/>
+    </row>
+    <row r="38" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="E38" s="30" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A39" s="13"/>
+      <c r="B39" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A40" s="37"/>
+      <c r="B40" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="19"/>
-    </row>
-    <row r="19" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="39"/>
-      <c r="B19" s="22" t="s">
+      <c r="D40" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="E40" s="18"/>
+    </row>
+    <row r="41" spans="1:5" ht="217.5" x14ac:dyDescent="0.35">
+      <c r="A41" s="37"/>
+      <c r="B41" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="E41" s="18"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A42" s="37"/>
+      <c r="B42" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E42" s="18"/>
+    </row>
+    <row r="43" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A43" s="37"/>
+      <c r="B43" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="E43" s="18"/>
+    </row>
+    <row r="44" spans="1:5" ht="391.5" x14ac:dyDescent="0.35">
+      <c r="A44" s="37"/>
+      <c r="B44" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="D44" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="E44" s="18"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A45" s="37"/>
+      <c r="B45" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="20"/>
+      <c r="D45" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="E45" s="18"/>
+    </row>
+    <row r="46" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A46" s="38"/>
+      <c r="B46" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="25"/>
-    </row>
-    <row r="20" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="B20" s="11" t="s">
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="24"/>
+    </row>
+    <row r="47" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A47" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B47" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="14"/>
-      <c r="B21" s="15" t="s">
+      <c r="C47" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E47" s="30"/>
+    </row>
+    <row r="48" spans="1:5" ht="116" x14ac:dyDescent="0.35">
+      <c r="A48" s="13"/>
+      <c r="B48" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="18"/>
-    </row>
-    <row r="22" spans="1:5" ht="116" x14ac:dyDescent="0.35">
-      <c r="A22" s="38"/>
-      <c r="B22" s="15" t="s">
+      <c r="C48" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="D48" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="E48" s="5"/>
+    </row>
+    <row r="49" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A49" s="37"/>
+      <c r="B49" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C22" s="28" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>71</v>
-      </c>
-      <c r="E22" s="19"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="38"/>
-      <c r="B23" s="17" t="s">
+      <c r="C49" s="27" t="s">
+        <v>98</v>
+      </c>
+      <c r="D49" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="E49" s="18"/>
+    </row>
+    <row r="50" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A50" s="37"/>
+      <c r="B50" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="C50" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="D50" s="33" t="s">
+        <v>105</v>
+      </c>
+      <c r="E50" s="18"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" s="37"/>
+      <c r="B51" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E51" s="18"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A52" s="37"/>
+      <c r="B52" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C52" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D52" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="E52" s="18"/>
+    </row>
+    <row r="53" spans="1:5" ht="87" x14ac:dyDescent="0.35">
+      <c r="A53" s="37"/>
+      <c r="B53" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C53" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="19"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="38"/>
-      <c r="B24" s="17" t="s">
+      <c r="D53" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="E53" s="18"/>
+    </row>
+    <row r="54" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A54" s="37"/>
+      <c r="B54" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C54" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="D54" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="E54" s="18"/>
+    </row>
+    <row r="55" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="38"/>
+      <c r="B55" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="C55" s="20"/>
+      <c r="D55" s="20"/>
+      <c r="E55" s="24"/>
+    </row>
+    <row r="56" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A56" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="E56" s="30"/>
+    </row>
+    <row r="57" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+      <c r="A57" s="13"/>
+      <c r="B57" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C57" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="D57" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="E57" s="5"/>
+    </row>
+    <row r="58" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="37"/>
+      <c r="B58" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C58" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="E58" s="18"/>
+    </row>
+    <row r="59" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A59" s="37"/>
+      <c r="B59" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C59" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D59" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="E59" s="18"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A60" s="37"/>
+      <c r="B60" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="19"/>
-    </row>
-    <row r="25" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A25" s="38"/>
-      <c r="B25" s="17" t="s">
+      <c r="E60" s="18"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="37"/>
+      <c r="B61" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="E25" s="19"/>
-    </row>
-    <row r="26" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A26" s="38"/>
-      <c r="B26" s="20" t="s">
+      <c r="C61" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="E61" s="18"/>
+    </row>
+    <row r="62" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A62" s="37"/>
+      <c r="B62" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="E26" s="19"/>
-    </row>
-    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="38"/>
-      <c r="B27" s="20" t="s">
+      <c r="C62" s="20"/>
+      <c r="D62" s="20" t="s">
+        <v>117</v>
+      </c>
+      <c r="E62" s="18"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A63" s="37"/>
+      <c r="B63" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="E27" s="19"/>
-    </row>
-    <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="39"/>
-      <c r="B28" s="22" t="s">
+      <c r="C63" s="20"/>
+      <c r="D63" s="32">
+        <v>0</v>
+      </c>
+      <c r="E63" s="18"/>
+    </row>
+    <row r="64" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="38"/>
+      <c r="B64" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="25"/>
-    </row>
-    <row r="29" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D29" s="35" t="s">
-        <v>123</v>
-      </c>
-      <c r="E29" s="31" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A30" s="14"/>
-      <c r="B30" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="D30" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A31" s="38"/>
-      <c r="B31" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D31" s="32" t="s">
-        <v>125</v>
-      </c>
-      <c r="E31" s="19"/>
-    </row>
-    <row r="32" spans="1:5" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A32" s="38"/>
-      <c r="B32" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="D32" s="32" t="s">
-        <v>126</v>
-      </c>
-      <c r="E32" s="19"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="38"/>
-      <c r="B33" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E33" s="19"/>
-    </row>
-    <row r="34" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A34" s="38"/>
-      <c r="B34" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D34" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="E34" s="19"/>
-    </row>
-    <row r="35" spans="1:5" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="A35" s="38"/>
-      <c r="B35" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="E35" s="19"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="38"/>
-      <c r="B36" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="21"/>
-      <c r="D36" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="E36" s="19"/>
-    </row>
-    <row r="37" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A37" s="39"/>
-      <c r="B37" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="25"/>
-    </row>
-    <row r="38" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A38" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" s="31" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A39" s="14"/>
-      <c r="B39" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="D39" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A40" s="38"/>
-      <c r="B40" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D40" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="E40" s="19"/>
-    </row>
-    <row r="41" spans="1:5" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="38"/>
-      <c r="B41" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="D41" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="E41" s="19"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="38"/>
-      <c r="B42" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E42" s="19"/>
-    </row>
-    <row r="43" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A43" s="38"/>
-      <c r="B43" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C43" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D43" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E43" s="19"/>
-    </row>
-    <row r="44" spans="1:5" ht="391.5" x14ac:dyDescent="0.35">
-      <c r="A44" s="38"/>
-      <c r="B44" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D44" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="E44" s="19"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="38"/>
-      <c r="B45" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C45" s="21"/>
-      <c r="D45" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="E45" s="19"/>
-    </row>
-    <row r="46" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A46" s="39"/>
-      <c r="B46" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="25"/>
-    </row>
-    <row r="47" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A47" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C47" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="D47" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="E47" s="31"/>
-    </row>
-    <row r="48" spans="1:5" ht="116" x14ac:dyDescent="0.35">
-      <c r="A48" s="14"/>
-      <c r="B48" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C48" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="D48" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="E48" s="6"/>
-    </row>
-    <row r="49" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A49" s="38"/>
-      <c r="B49" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C49" s="28" t="s">
-        <v>99</v>
-      </c>
-      <c r="D49" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="E49" s="19"/>
-    </row>
-    <row r="50" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A50" s="38"/>
-      <c r="B50" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C50" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="D50" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="E50" s="19"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="38"/>
-      <c r="B51" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E51" s="19"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="38"/>
-      <c r="B52" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C52" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D52" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="E52" s="19"/>
-    </row>
-    <row r="53" spans="1:5" ht="87" x14ac:dyDescent="0.35">
-      <c r="A53" s="38"/>
-      <c r="B53" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C53" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="D53" s="21" t="s">
-        <v>105</v>
-      </c>
-      <c r="E53" s="19"/>
-    </row>
-    <row r="54" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A54" s="38"/>
-      <c r="B54" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C54" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="D54" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="E54" s="19"/>
-    </row>
-    <row r="55" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A55" s="39"/>
-      <c r="B55" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C55" s="21"/>
-      <c r="D55" s="21"/>
-      <c r="E55" s="25"/>
-    </row>
-    <row r="56" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A56" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="B56" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C56" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="D56" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="E56" s="31"/>
-    </row>
-    <row r="57" spans="1:5" ht="58" x14ac:dyDescent="0.35">
-      <c r="A57" s="14"/>
-      <c r="B57" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="C57" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="D57" s="28" t="s">
-        <v>114</v>
-      </c>
-      <c r="E57" s="6"/>
-    </row>
-    <row r="58" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A58" s="38"/>
-      <c r="B58" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C58" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D58" s="34" t="s">
-        <v>115</v>
-      </c>
-      <c r="E58" s="19"/>
-    </row>
-    <row r="59" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A59" s="38"/>
-      <c r="B59" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C59" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D59" s="34" t="s">
-        <v>116</v>
-      </c>
-      <c r="E59" s="19"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" s="38"/>
-      <c r="B60" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="E60" s="19"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" s="38"/>
-      <c r="B61" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C61" s="28" t="s">
-        <v>42</v>
-      </c>
-      <c r="D61" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="E61" s="19"/>
-    </row>
-    <row r="62" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A62" s="38"/>
-      <c r="B62" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C62" s="21"/>
-      <c r="D62" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="E62" s="19"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" s="38"/>
-      <c r="B63" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C63" s="21"/>
-      <c r="D63" s="33">
-        <v>0</v>
-      </c>
-      <c r="E63" s="19"/>
-    </row>
-    <row r="64" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A64" s="39"/>
-      <c r="B64" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="C64" s="21"/>
-      <c r="D64" s="21"/>
-      <c r="E64" s="25"/>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>